<commit_message>
Modification du tableau de synthèse et ajout du chemin pour la situation professionelle 1 et ajout du contrat de developpement absent
</commit_message>
<xml_diff>
--- a/documents/tableau_synthèse.xlsx
+++ b/documents/tableau_synthèse.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\enzog\OneDrive\Desktop\Projet informatique programation etc\portfolio\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6D2694-414B-4FA3-88A8-70A22DD289DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8603F13B-F222-4C32-9DE8-8884C6026D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$21</definedName>
   </definedNames>
   <calcPr calcId="181029" concurrentCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="35">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -122,9 +122,6 @@
     <t>Mise en place de la veille technologique, du profil professionnel et des besoins en formation(carte heuristique d'un métier, portfolio, veille technologique, profil LinkedIn, pearltree de formations)</t>
   </si>
   <si>
-    <t>SESSION 2025</t>
-  </si>
-  <si>
     <t>AP1 : évolution dun site web (Symfony) avec qualité de code, accès avec authentification, tests unitaire et fonctionnels, mise en ligne du site, de la BDD : mise à disposition des formations  de la médiathèque Mediatek86 (code source, BDD, tests unitaires et fonctionnels, documentation technique, documentation utilisateur)</t>
   </si>
   <si>
@@ -144,6 +141,12 @@
   </si>
   <si>
     <t>Développement d'une nouvelle application et correction de problème dans un logiciel déjà éxistant.</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://0mega15.github.io/portfolio/index.html</t>
+  </si>
+  <si>
+    <t>SESSION 2026</t>
   </si>
 </sst>
 </file>
@@ -226,7 +229,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -422,9 +425,31 @@
       <right style="thin">
         <color theme="2" tint="-0.749992370372631"/>
       </right>
-      <top style="medium">
+      <top/>
+      <bottom style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
         <color theme="2" tint="-0.749992370372631"/>
       </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -436,8 +461,34 @@
         <color theme="2" tint="-0.749992370372631"/>
       </right>
       <top/>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -446,7 +497,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -460,15 +511,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -496,9 +538,36 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -508,35 +577,29 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -846,7 +909,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ66"/>
+  <dimension ref="A1:AQ67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
@@ -857,160 +920,125 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
     </row>
     <row r="3" spans="1:43" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="18" t="s">
+      <c r="A3" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="19"/>
-      <c r="H3" s="20"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="26"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="40.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="18" t="s">
+    <row r="4" spans="1:43" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="10" t="s">
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
+    <row r="5" spans="1:43" ht="40.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="34"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B6" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C6" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D6" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E6" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F6" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G6" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H6" s="30" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:43" s="2" customFormat="1" ht="325.35000000000002" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
-      <c r="B6" s="30"/>
-      <c r="C6" s="14" t="s">
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="325.35000000000002" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="15"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D7" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F7" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G7" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="H7" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="I6"/>
-      <c r="J6"/>
-      <c r="K6"/>
-      <c r="L6"/>
-      <c r="M6"/>
-      <c r="N6"/>
-      <c r="O6"/>
-      <c r="P6"/>
-      <c r="Q6"/>
-      <c r="R6"/>
-      <c r="S6"/>
-      <c r="T6"/>
-      <c r="U6"/>
-      <c r="V6"/>
-      <c r="W6"/>
-      <c r="X6"/>
-      <c r="Y6"/>
-      <c r="Z6"/>
-      <c r="AA6"/>
-      <c r="AB6"/>
-      <c r="AC6"/>
-      <c r="AD6"/>
-      <c r="AE6"/>
-      <c r="AF6"/>
-      <c r="AG6"/>
-      <c r="AH6"/>
-      <c r="AI6"/>
-      <c r="AJ6"/>
-      <c r="AK6"/>
-      <c r="AL6"/>
-      <c r="AM6"/>
-      <c r="AN6"/>
-      <c r="AO6"/>
-      <c r="AP6"/>
-      <c r="AQ6"/>
-    </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A7" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="25"/>
       <c r="I7"/>
       <c r="J7"/>
       <c r="K7"/>
@@ -1047,19 +1075,17 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="13" t="s">
-        <v>23</v>
-      </c>
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="19"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1096,15 +1122,19 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="13"/>
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="10" t="s">
+        <v>23</v>
+      </c>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1141,27 +1171,15 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="69" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" s="13"/>
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A10" s="6"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="10"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1198,25 +1216,27 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="82.8" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" s="13"/>
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="69" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" s="10"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1253,15 +1273,25 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="13"/>
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="82.8" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H12" s="10"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1298,17 +1328,15 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A13" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="28"/>
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A13" s="6"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="10"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1345,21 +1373,17 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G14" s="12"/>
-      <c r="H14" s="13"/>
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A14" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="22"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1396,15 +1420,21 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="13"/>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" s="9"/>
+      <c r="H15" s="10"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1441,17 +1471,15 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A16" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="28"/>
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A16" s="6"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="10"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1488,19 +1516,17 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="13"/>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A17" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="22"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1537,23 +1563,19 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="H18" s="13"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="10"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1590,25 +1612,23 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="H19" s="13"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H19" s="10"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1646,14 +1666,24 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A20" s="5"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
+      <c r="A20" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H20" s="10"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1690,8 +1720,54 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A21"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21"/>
+      <c r="J21"/>
+      <c r="K21"/>
+      <c r="L21"/>
+      <c r="M21"/>
+      <c r="N21"/>
+      <c r="O21"/>
+      <c r="P21"/>
+      <c r="Q21"/>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+      <c r="U21"/>
+      <c r="V21"/>
+      <c r="W21"/>
+      <c r="X21"/>
+      <c r="Y21"/>
+      <c r="Z21"/>
+      <c r="AA21"/>
+      <c r="AB21"/>
+      <c r="AC21"/>
+      <c r="AD21"/>
+      <c r="AE21"/>
+      <c r="AF21"/>
+      <c r="AG21"/>
+      <c r="AH21"/>
+      <c r="AI21"/>
+      <c r="AJ21"/>
+      <c r="AK21"/>
+      <c r="AL21"/>
+      <c r="AM21"/>
+      <c r="AN21"/>
+      <c r="AO21"/>
+      <c r="AP21"/>
+      <c r="AQ21"/>
+    </row>
+    <row r="22" spans="1:43" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+    </row>
     <row r="23" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="24" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -1736,19 +1812,20 @@
     <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="B5:B6"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="F3:H3"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="B6:B7"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>

<commit_message>
Mise à jour des dates dans le tableau de synthèse
</commit_message>
<xml_diff>
--- a/documents/tableau_synthèse.xlsx
+++ b/documents/tableau_synthèse.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\enzog\OneDrive\Desktop\Projet informatique programation etc\portfolio\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8603F13B-F222-4C32-9DE8-8884C6026D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAA93BC1-CEA1-4BB8-9590-106DA93692B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="40">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -147,6 +147,21 @@
   </si>
   <si>
     <t>SESSION 2026</t>
+  </si>
+  <si>
+    <t>16/09/2025 au 01/05/2026</t>
+  </si>
+  <si>
+    <t>05/01/2026 au 30/03/2026</t>
+  </si>
+  <si>
+    <t>23/03/2026 au 02/05/2026</t>
+  </si>
+  <si>
+    <t>24/03/2025 au 25/04/2025</t>
+  </si>
+  <si>
+    <t>19/01/2026 au 20/02/2026</t>
   </si>
 </sst>
 </file>
@@ -497,7 +512,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -600,6 +615,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -913,7 +934,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.77734375" style="1" customWidth="1"/>
     <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
     <col min="9" max="43" width="11.44140625" customWidth="1"/>
     <col min="44" max="16384" width="10.6640625" style="1"/>
@@ -1126,7 +1147,9 @@
       <c r="A9" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="5"/>
+      <c r="B9" s="35" t="s">
+        <v>35</v>
+      </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
@@ -1220,7 +1243,9 @@
       <c r="A11" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="5"/>
+      <c r="B11" s="36" t="s">
+        <v>36</v>
+      </c>
       <c r="C11" s="9" t="s">
         <v>23</v>
       </c>
@@ -1277,7 +1302,9 @@
       <c r="A12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="5"/>
+      <c r="B12" s="36" t="s">
+        <v>37</v>
+      </c>
       <c r="C12" s="9" t="s">
         <v>23</v>
       </c>
@@ -1420,11 +1447,13 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="5"/>
+      <c r="B15" s="36" t="s">
+        <v>38</v>
+      </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9" t="s">
         <v>23</v>
@@ -1563,11 +1592,13 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="5"/>
+      <c r="B18" s="36" t="s">
+        <v>39</v>
+      </c>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9" t="s">
@@ -1612,11 +1643,13 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="5"/>
+      <c r="B19" s="36" t="s">
+        <v>39</v>
+      </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9" t="s">
         <v>23</v>
@@ -1665,11 +1698,13 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="5"/>
+      <c r="B20" s="36" t="s">
+        <v>39</v>
+      </c>
       <c r="C20" s="9" t="s">
         <v>23</v>
       </c>
@@ -1830,7 +1865,7 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="45" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="52" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout de la page mediatekDocument et des éléments
</commit_message>
<xml_diff>
--- a/documents/tableau_synthèse.xlsx
+++ b/documents/tableau_synthèse.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\enzog\OneDrive\Desktop\Projet informatique programation etc\portfolio\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAA93BC1-CEA1-4BB8-9590-106DA93692B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FAE436-D688-4754-A26D-EC4974E147EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -101,9 +101,6 @@
 (intitulé et liste des documents et productions associés)</t>
   </si>
   <si>
-    <t xml:space="preserve">N° candidat : </t>
-  </si>
-  <si>
     <t>Période (sous la forme du JJ/MM/AA au JJ/MM/AA)</t>
   </si>
   <si>
@@ -162,6 +159,9 @@
   </si>
   <si>
     <t>19/01/2026 au 20/02/2026</t>
+  </si>
+  <si>
+    <t>N° candidat : 02249594168</t>
   </si>
 </sst>
 </file>
@@ -553,15 +553,51 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -580,47 +616,11 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -941,41 +941,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="H1" s="16"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
     </row>
     <row r="3" spans="1:43" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B3" s="25"/>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
       <c r="E3" s="26"/>
       <c r="F3" s="24" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="G3" s="25"/>
       <c r="H3" s="26"/>
@@ -985,7 +985,7 @@
     </row>
     <row r="4" spans="1:43" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" s="25"/>
       <c r="C4" s="25"/>
@@ -1002,46 +1002,46 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="40.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="34"/>
+      <c r="A5" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="29" t="s">
+      <c r="B6" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="29" t="s">
+      <c r="F6" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="29" t="s">
+      <c r="G6" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="16" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325.35000000000002" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="15"/>
-      <c r="B7" s="23"/>
+      <c r="A7" s="28"/>
+      <c r="B7" s="36"/>
       <c r="C7" s="11" t="s">
         <v>9</v>
       </c>
@@ -1097,16 +1097,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="19"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="31"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1145,10 +1145,10 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="35" t="s">
-        <v>35</v>
+        <v>24</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>34</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
@@ -1156,7 +1156,7 @@
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
       <c r="H9" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I9"/>
       <c r="J9"/>
@@ -1241,25 +1241,25 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="69" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="36" t="s">
-        <v>36</v>
+        <v>25</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>35</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H11" s="10"/>
       <c r="I11"/>
@@ -1300,23 +1300,23 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="82.8" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="36" t="s">
-        <v>37</v>
+        <v>26</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>36</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E12" s="9"/>
       <c r="F12" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H12" s="10"/>
       <c r="I12"/>
@@ -1401,16 +1401,16 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A14" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="22"/>
+      <c r="A14" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="33"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="34"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1449,18 +1449,18 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="36" t="s">
-        <v>38</v>
+        <v>31</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>37</v>
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G15" s="9"/>
       <c r="H15" s="10"/>
@@ -1546,16 +1546,16 @@
       <c r="AQ16"/>
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A17" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="22"/>
+      <c r="A17" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="34"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1594,15 +1594,15 @@
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="36" t="s">
-        <v>39</v>
+        <v>30</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>38</v>
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
@@ -1645,21 +1645,21 @@
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="36" t="s">
-        <v>39</v>
+        <v>29</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>38</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E19" s="9"/>
       <c r="F19" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H19" s="10"/>
       <c r="I19"/>
@@ -1700,23 +1700,23 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="36" t="s">
-        <v>39</v>
+        <v>28</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>38</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H20" s="10"/>
       <c r="I20"/>
@@ -1850,17 +1850,17 @@
     <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="B6:B7"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>